<commit_message>
Add 3 new note.com articles (Esse STEP16/STEP28-0, HP announcement)
Sync data/note_articles_metadata.xlsx and regenerate content/articles/note
stubs from the latest note.com posts. Also track Note記事一覧.xlsx (STEP x
car-model coverage matrix) and ignore Office lock files.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/note_articles_metadata.xlsx
+++ b/data/note_articles_metadata.xlsx
@@ -128,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -147,6 +147,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -731,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M294"/>
+  <dimension ref="A1:M297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -18003,6 +18004,189 @@
       </c>
       <c r="M294" s="5" t="n">
         <v>300</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="12" t="inlineStr">
+        <is>
+          <t>esse-linkecu-step16-0a8823</t>
+        </is>
+      </c>
+      <c r="B295" s="12" t="inlineStr">
+        <is>
+          <t>エッセ KF-VE LINKECU フルコン化 STEP16 デジタルインプット ブレーキスイッチ 信号入力</t>
+        </is>
+      </c>
+      <c r="C295" s="12" t="inlineStr">
+        <is>
+          <t>エッセ(ESSE)</t>
+        </is>
+      </c>
+      <c r="D295" s="12" t="inlineStr">
+        <is>
+          <t>LINKECU</t>
+        </is>
+      </c>
+      <c r="E295" s="12" t="inlineStr">
+        <is>
+          <t>エッセをLINKECUでフルコン化していきます。今回はブレーキON信号をECUに入力します。</t>
+        </is>
+      </c>
+      <c r="F295" s="12" t="inlineStr">
+        <is>
+          <t>https://note.com/labratory_ktech/n/n00ea3a0a8823</t>
+        </is>
+      </c>
+      <c r="G295" s="12" t="inlineStr">
+        <is>
+          <t>esse-linkecu-step15-528668, esse-linkecu-step17-3-07f585</t>
+        </is>
+      </c>
+      <c r="H295" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="I295" s="12" t="inlineStr">
+        <is>
+          <t>STEP本編（フルコン化手順）</t>
+        </is>
+      </c>
+      <c r="J295" s="12" t="inlineStr">
+        <is>
+          <t>STEP16</t>
+        </is>
+      </c>
+      <c r="K295" s="12" t="inlineStr">
+        <is>
+          <t>エッセ ESSE LINKECU フルコン化 への道</t>
+        </is>
+      </c>
+      <c r="L295" s="12" t="inlineStr">
+        <is>
+          <t>#入力 #ブレーキ #エッセ #LINKECU #フルコン化 #デジタルインプット #ブレーキスイッチ #信号入力 #Step16</t>
+        </is>
+      </c>
+      <c r="M295" s="12" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="12" t="inlineStr">
+        <is>
+          <t>esse-linkecu-step28-0-914ffb</t>
+        </is>
+      </c>
+      <c r="B296" s="12" t="inlineStr">
+        <is>
+          <t>エッセ LINKECU化への道 STEP28-0 VVT制御 ソレノイド PWM周波数 調査結果</t>
+        </is>
+      </c>
+      <c r="C296" s="12" t="inlineStr">
+        <is>
+          <t>エッセ(ESSE)</t>
+        </is>
+      </c>
+      <c r="D296" s="12" t="inlineStr">
+        <is>
+          <t>LINKECU</t>
+        </is>
+      </c>
+      <c r="E296" s="12" t="inlineStr">
+        <is>
+          <t>エッセの純正ECUがVVTソレノイドを駆動しているPWM周波数を実測し、LINKECU化時の初期設定値の目安を紹介します。</t>
+        </is>
+      </c>
+      <c r="F296" s="12" t="inlineStr">
+        <is>
+          <t>https://note.com/labratory_ktech/n/n77f803914ffb</t>
+        </is>
+      </c>
+      <c r="G296" s="12" t="inlineStr">
+        <is>
+          <t>esse-linkecu-step27-2-2e1dbc</t>
+        </is>
+      </c>
+      <c r="H296" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="I296" s="12" t="inlineStr">
+        <is>
+          <t>STEP本編（フルコン化手順）</t>
+        </is>
+      </c>
+      <c r="J296" s="12" t="inlineStr">
+        <is>
+          <t>STEP28-0</t>
+        </is>
+      </c>
+      <c r="K296" s="12" t="inlineStr">
+        <is>
+          <t>エッセ ESSE LINKECU フルコン化 への道</t>
+        </is>
+      </c>
+      <c r="L296" s="12" t="inlineStr">
+        <is>
+          <t>#調査結果 #エッセ #ソレノイド #PWM周波数 #LINKECU化への道 #VVT制御</t>
+        </is>
+      </c>
+      <c r="M296" s="12" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="12" t="inlineStr">
+        <is>
+          <t>misc-linkindex-7b23f2</t>
+        </is>
+      </c>
+      <c r="B297" s="12" t="inlineStr">
+        <is>
+          <t>Note記事検索用 HP作成しました</t>
+        </is>
+      </c>
+      <c r="C297" s="12" t="inlineStr">
+        <is>
+          <t>（共通・車種特定なし）</t>
+        </is>
+      </c>
+      <c r="D297" s="12" t="n"/>
+      <c r="E297" s="12" t="inlineStr">
+        <is>
+          <t>note.comの記事が増え検索性が課題になったため、記事・マガジン単位で整理し全文検索できる専用HP（kim23-lab-index）を作成しました。</t>
+        </is>
+      </c>
+      <c r="F297" s="12" t="inlineStr">
+        <is>
+          <t>https://note.com/labratory_ktech/n/n224cad7b23f2</t>
+        </is>
+      </c>
+      <c r="G297" s="12" t="n"/>
+      <c r="H297" s="12" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="I297" s="12" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="J297" s="12" t="n"/>
+      <c r="K297" s="12" t="inlineStr">
+        <is>
+          <t>LINKECU 関連/技術資料LINK集</t>
+        </is>
+      </c>
+      <c r="L297" s="12" t="inlineStr">
+        <is>
+          <t>#Link #リンク集 #検索用</t>
+        </is>
+      </c>
+      <c r="M297" s="12" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mark MaxxECU power-supply and PWM articles as free
Both articles are now free on note.com; sync price to 0 in the
article stubs and in the source metadata xlsx so re-importing keeps it.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/note_articles_metadata.xlsx
+++ b/data/note_articles_metadata.xlsx
@@ -4783,7 +4783,7 @@
         </is>
       </c>
       <c r="M70" s="5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -6332,7 +6332,7 @@
         </is>
       </c>
       <c r="M95" s="5" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">

</xml_diff>

<commit_message>
Add 5 new note.com articles (pull-up reverse calc, Esse STEP28-1, etc.)
Sync data/note_articles_metadata.xlsx with the posts from 2026-10-07 to
2026-10-18 and regenerate the note stubs: pull-up resistor reverse
calculation, Esse STEP28-1 VVT wiring, Sonica fuel pump flow, Paint AI
erase, and the smartphone + Wi-Fi camera GPS log (VER0). STEP28-0 now
links to STEP28-1, and the ArticleMetadata table range covers all rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/note_articles_metadata.xlsx
+++ b/data/note_articles_metadata.xlsx
@@ -225,8 +225,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ArticleMetadata" displayName="ArticleMetadata" ref="A1:M294" headerRowCount="1">
-  <autoFilter ref="A1:M294"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ArticleMetadata" displayName="ArticleMetadata" ref="A1:M302" headerRowCount="1">
+  <autoFilter ref="A1:M302"/>
   <tableColumns count="13">
     <tableColumn id="1" name="slug"/>
     <tableColumn id="2" name="title"/>
@@ -732,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M297"/>
+  <dimension ref="A1:M302"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -18104,7 +18104,7 @@
       </c>
       <c r="G296" s="12" t="inlineStr">
         <is>
-          <t>esse-linkecu-step27-2-2e1dbc</t>
+          <t>esse-linkecu-step27-2-2e1dbc, esse-linkecu-step28-1-9587f7</t>
         </is>
       </c>
       <c r="H296" s="12" t="inlineStr">
@@ -18186,6 +18186,299 @@
         </is>
       </c>
       <c r="M297" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="12" t="inlineStr">
+        <is>
+          <t>misc-88bf2d</t>
+        </is>
+      </c>
+      <c r="B298" s="12" t="inlineStr">
+        <is>
+          <t>スマホとWi‑Fiカメラだけで動画付きGPSログを作る（VER0）</t>
+        </is>
+      </c>
+      <c r="C298" s="12" t="inlineStr">
+        <is>
+          <t>（共通・車種特定なし）</t>
+        </is>
+      </c>
+      <c r="D298" s="12" t="n"/>
+      <c r="E298" s="12" t="inlineStr">
+        <is>
+          <t>スマホのGPSとWi-Fiカメラ（M5Stack UnitV2）を組み合わせて、動画付きのGPS走行ログを作るVER0の構成を紹介します。</t>
+        </is>
+      </c>
+      <c r="F298" s="12" t="inlineStr">
+        <is>
+          <t>https://note.com/labratory_ktech/n/nc2ef1688bf2d</t>
+        </is>
+      </c>
+      <c r="G298" s="12" t="inlineStr">
+        <is>
+          <t>misc-linkecu-0a5a37</t>
+        </is>
+      </c>
+      <c r="H298" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="I298" s="12" t="inlineStr">
+        <is>
+          <t>電子工作・自作ツール</t>
+        </is>
+      </c>
+      <c r="J298" s="12" t="n"/>
+      <c r="K298" s="12" t="inlineStr">
+        <is>
+          <t>パーツレビュー/データロガービューアー製作</t>
+        </is>
+      </c>
+      <c r="L298" s="12" t="inlineStr">
+        <is>
+          <t>#カメラ #スマホ #電子工作 #wifi #動画撮影 #GPS #CAN #データロガー #GPSロガー</t>
+        </is>
+      </c>
+      <c r="M298" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="12" t="inlineStr">
+        <is>
+          <t>misc-e9a9fd</t>
+        </is>
+      </c>
+      <c r="B299" s="12" t="inlineStr">
+        <is>
+          <t>Windows標準のペイントに AI削除機能があったので使ってみたら、思った以上に使えました</t>
+        </is>
+      </c>
+      <c r="C299" s="12" t="inlineStr">
+        <is>
+          <t>（共通・車種特定なし）</t>
+        </is>
+      </c>
+      <c r="D299" s="12" t="n"/>
+      <c r="E299" s="12" t="inlineStr">
+        <is>
+          <t>Windows標準のペイントにある「生成消去」（AI削除）機能で、写真の不要な写り込みを消してみました。</t>
+        </is>
+      </c>
+      <c r="F299" s="12" t="inlineStr">
+        <is>
+          <t>https://note.com/labratory_ktech/n/n19620fe9a9fd</t>
+        </is>
+      </c>
+      <c r="G299" s="12" t="n"/>
+      <c r="H299" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="I299" s="12" t="inlineStr">
+        <is>
+          <t>その他</t>
+        </is>
+      </c>
+      <c r="J299" s="12" t="n"/>
+      <c r="K299" s="12" t="inlineStr">
+        <is>
+          <t>画像編集関連</t>
+        </is>
+      </c>
+      <c r="L299" s="12" t="inlineStr">
+        <is>
+          <t>#AI #簡単 #画像生成 #ソフト #画像編集 #ペイント #paint</t>
+        </is>
+      </c>
+      <c r="M299" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="12" t="inlineStr">
+        <is>
+          <t>esse-linkecu-step28-1-9587f7</t>
+        </is>
+      </c>
+      <c r="B300" s="12" t="inlineStr">
+        <is>
+          <t>エッセ LINKECU化 STEP28-1 KF-VE VVT 配線 を調べてみたOCV+って何？ OCV-って何？</t>
+        </is>
+      </c>
+      <c r="C300" s="12" t="inlineStr">
+        <is>
+          <t>エッセ(ESSE)</t>
+        </is>
+      </c>
+      <c r="D300" s="12" t="inlineStr">
+        <is>
+          <t>LINKECU</t>
+        </is>
+      </c>
+      <c r="E300" s="12" t="inlineStr">
+        <is>
+          <t>エッセ KF-VE の純正配線図にあるVVTのOCV+ / OCV−が、実際にどちら側をECUが制御しているのかを調べ、LINKECUへ移植するときの配線を確認します。</t>
+        </is>
+      </c>
+      <c r="F300" s="12" t="inlineStr">
+        <is>
+          <t>https://note.com/labratory_ktech/n/nc5e7ee9587f7</t>
+        </is>
+      </c>
+      <c r="G300" s="12" t="inlineStr">
+        <is>
+          <t>esse-linkecu-step28-0-914ffb</t>
+        </is>
+      </c>
+      <c r="H300" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="I300" s="12" t="inlineStr">
+        <is>
+          <t>STEP本編（フルコン化手順）</t>
+        </is>
+      </c>
+      <c r="J300" s="12" t="inlineStr">
+        <is>
+          <t>STEP28-1</t>
+        </is>
+      </c>
+      <c r="K300" s="12" t="inlineStr">
+        <is>
+          <t>LINKECU 関連/ECUフルコン化への道/エッセ ESSE LINKECU フルコン化 への道</t>
+        </is>
+      </c>
+      <c r="L300" s="12" t="inlineStr">
+        <is>
+          <t>#確認 #出力 #制御 #配線 #純正 #電圧 #エッセ #LINKECU化 #VVT</t>
+        </is>
+      </c>
+      <c r="M300" s="12" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="12" t="inlineStr">
+        <is>
+          <t>sonica-c2d14c</t>
+        </is>
+      </c>
+      <c r="B301" s="12" t="inlineStr">
+        <is>
+          <t>ソニカ KF-DET 純正燃料ポンプ 流量 を実測してみた　ブーストアップ時 の ボトルネックを把握する</t>
+        </is>
+      </c>
+      <c r="C301" s="12" t="inlineStr">
+        <is>
+          <t>ソニカ(SONICA)</t>
+        </is>
+      </c>
+      <c r="D301" s="12" t="n"/>
+      <c r="E301" s="12" t="inlineStr">
+        <is>
+          <t>ソニカ KF-DET の純正燃料ポンプの流量を実測し、ブーストアップ時に純正ポンプで支えられる馬力を計算します。</t>
+        </is>
+      </c>
+      <c r="F301" s="12" t="inlineStr">
+        <is>
+          <t>https://note.com/labratory_ktech/n/n0513dbc2d14c</t>
+        </is>
+      </c>
+      <c r="G301" s="12" t="inlineStr">
+        <is>
+          <t>sonica-2705aa, altoworks-linkecu-e70d48, altoworks-59ffdc</t>
+        </is>
+      </c>
+      <c r="H301" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="I301" s="12" t="inlineStr">
+        <is>
+          <t>部品選定・レビュー</t>
+        </is>
+      </c>
+      <c r="J301" s="12" t="n"/>
+      <c r="K301" s="12" t="inlineStr">
+        <is>
+          <t>エッセ ESSE LINKECU フルコン化 への道/ソニカ KF-DET フルコン化/パーツレビュー/燃料、インジェクター関連 無効噴射時間</t>
+        </is>
+      </c>
+      <c r="L301" s="12" t="inlineStr">
+        <is>
+          <t>#実験結果 #流量 #燃料ポンプ #ソニカ #実測結果 #純正燃料ポンプ</t>
+        </is>
+      </c>
+      <c r="M301" s="12" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="12" t="inlineStr">
+        <is>
+          <t>misc-linkecu-8674a0</t>
+        </is>
+      </c>
+      <c r="B302" s="12" t="inlineStr">
+        <is>
+          <t>ECUフルコン化への道 抵抗1本でECUのプルアップ抵抗を逆算する方法　HPに計算ツール追加</t>
+        </is>
+      </c>
+      <c r="C302" s="12" t="inlineStr">
+        <is>
+          <t>（共通・車種特定なし）</t>
+        </is>
+      </c>
+      <c r="D302" s="12" t="inlineStr">
+        <is>
+          <t>LINKECU</t>
+        </is>
+      </c>
+      <c r="E302" s="12" t="inlineStr">
+        <is>
+          <t>抵抗を1本つないでECU入力電圧を測るだけで、純正ECU内部のプルアップ抵抗値を逆算する方法を紹介します。HPに計算ツールも追加しました。</t>
+        </is>
+      </c>
+      <c r="F302" s="12" t="inlineStr">
+        <is>
+          <t>https://note.com/labratory_ktech/n/ncde3d68674a0</t>
+        </is>
+      </c>
+      <c r="G302" s="12" t="inlineStr">
+        <is>
+          <t>altoworks-b01abe, misc-a2b1f2</t>
+        </is>
+      </c>
+      <c r="H302" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="I302" s="12" t="inlineStr">
+        <is>
+          <t>センサ・計測データ</t>
+        </is>
+      </c>
+      <c r="J302" s="12" t="n"/>
+      <c r="K302" s="12" t="inlineStr">
+        <is>
+          <t>温度センサ関連/LINKECU 関連/ECUフルコン化への道</t>
+        </is>
+      </c>
+      <c r="L302" s="12" t="inlineStr">
+        <is>
+          <t>#抵抗 #計算式 #電圧 #センサ #抵抗値 #プルアップ #ECUフルコン化への道 #抵抗1本でECUのプルアップ抵抗を逆算する方法</t>
+        </is>
+      </c>
+      <c r="M302" s="12" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>